<commit_message>
GL+CP more fields added
</commit_message>
<xml_diff>
--- a/src/data/property_lob.xlsx
+++ b/src/data/property_lob.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mudita\Documents\spg-automation\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718344F4-C41D-4AE4-BEB0-DE51B55869AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF3D722-EC99-40FF-86F7-F6F4C78BBBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Policy_Info" sheetId="1" r:id="rId1"/>
@@ -24,6 +24,9 @@
     <sheet name="GL_ClassCodes_Atrium" sheetId="4" r:id="rId9"/>
     <sheet name="GL_AddlInsureds" sheetId="7" r:id="rId10"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">CP_OccupancyQ!$A$1:$FA$30</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13407" uniqueCount="2733">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13408" uniqueCount="2733">
   <si>
     <t>Test ID</t>
   </si>
@@ -8303,7 +8306,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -8325,6 +8328,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -8369,7 +8384,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -8411,6 +8426,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8946,16 +8966,16 @@
       <c r="BA1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BB1" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BC1" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BD1" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BE1" s="25" t="s">
         <v>56</v>
       </c>
       <c r="BF1" s="3"/>
@@ -24612,6 +24632,44 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA1A6362-89C5-4D93-8832-E7F9BBB0A69F}">
   <dimension ref="A1:AK37"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="20.21875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="29.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="17.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:37">
       <c r="A1" t="s">
@@ -24620,43 +24678,43 @@
       <c r="B1" t="s">
         <v>1072</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="26" t="s">
         <v>1073</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="26" t="s">
         <v>1074</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="26" t="s">
         <v>1075</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="26" t="s">
         <v>1076</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="26" t="s">
         <v>1077</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="26" t="s">
         <v>1078</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="26" t="s">
         <v>1079</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="26" t="s">
         <v>1080</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="26" t="s">
         <v>1081</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="26" t="s">
         <v>1082</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="26" t="s">
         <v>1083</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="26" t="s">
         <v>1084</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="26" t="s">
         <v>1085</v>
       </c>
       <c r="P1" t="s">
@@ -24683,31 +24741,31 @@
       <c r="W1" t="s">
         <v>1093</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="26" t="s">
         <v>1094</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="26" t="s">
         <v>1095</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="26" t="s">
         <v>1096</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="26" t="s">
         <v>1097</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="26" t="s">
         <v>1098</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="26" t="s">
         <v>1099</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="26" t="s">
         <v>1100</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="26" t="s">
         <v>1101</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="26" t="s">
         <v>1102</v>
       </c>
       <c r="AG1" t="s">
@@ -27905,6 +27963,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -28397,31 +28456,31 @@
       <c r="DD1" t="s">
         <v>1386</v>
       </c>
-      <c r="DE1" t="s">
+      <c r="DE1" s="26" t="s">
         <v>1387</v>
       </c>
-      <c r="DF1" t="s">
+      <c r="DF1" s="26" t="s">
         <v>1388</v>
       </c>
-      <c r="DG1" t="s">
+      <c r="DG1" s="26" t="s">
         <v>1389</v>
       </c>
-      <c r="DH1" t="s">
+      <c r="DH1" s="26" t="s">
         <v>1390</v>
       </c>
       <c r="DI1" t="s">
         <v>1391</v>
       </c>
-      <c r="DJ1" t="s">
+      <c r="DJ1" s="26" t="s">
         <v>1392</v>
       </c>
-      <c r="DK1" t="s">
+      <c r="DK1" s="26" t="s">
         <v>1393</v>
       </c>
-      <c r="DL1" t="s">
+      <c r="DL1" s="26" t="s">
         <v>1394</v>
       </c>
-      <c r="DM1" t="s">
+      <c r="DM1" s="26" t="s">
         <v>1395</v>
       </c>
       <c r="DN1" t="s">
@@ -42263,16 +42322,32 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:FA30" xr:uid="{FFAC7337-2B0D-48A6-8A09-24DFDC33FFCD}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5F37BAF-63A8-405D-8DF2-6BEC3B2C8934}">
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.88671875" customWidth="1"/>
+    <col min="13" max="13" width="49.5546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -42306,11 +42381,14 @@
       <c r="K1" t="s">
         <v>2041</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="27" t="s">
+        <v>1085</v>
+      </c>
+      <c r="M1" t="s">
         <v>795</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -42344,11 +42422,11 @@
       <c r="K2" t="s">
         <v>60</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>808</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>89</v>
       </c>
@@ -42382,11 +42460,11 @@
       <c r="K3" t="s">
         <v>59</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>813</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
         <v>121</v>
       </c>
@@ -42420,11 +42498,11 @@
       <c r="K4" t="s">
         <v>59</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>826</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
         <v>150</v>
       </c>
@@ -42458,11 +42536,11 @@
       <c r="K5" t="s">
         <v>60</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>818</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
         <v>174</v>
       </c>
@@ -42496,11 +42574,11 @@
       <c r="K6" t="s">
         <v>59</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
         <v>188</v>
       </c>
@@ -42534,11 +42612,11 @@
       <c r="K7" t="s">
         <v>60</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>826</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
         <v>210</v>
       </c>
@@ -42572,11 +42650,11 @@
       <c r="K8" t="s">
         <v>59</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>829</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
         <v>229</v>
       </c>
@@ -42610,11 +42688,11 @@
       <c r="K9" t="s">
         <v>60</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>826</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
         <v>252</v>
       </c>
@@ -42648,11 +42726,11 @@
       <c r="K10" t="s">
         <v>60</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
         <v>274</v>
       </c>
@@ -42686,11 +42764,11 @@
       <c r="K11" t="s">
         <v>60</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="12" spans="1:12">
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
         <v>295</v>
       </c>
@@ -42724,11 +42802,11 @@
       <c r="K12" t="s">
         <v>60</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
         <v>315</v>
       </c>
@@ -42762,11 +42840,11 @@
       <c r="K13" t="s">
         <v>60</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
         <v>336</v>
       </c>
@@ -42800,11 +42878,11 @@
       <c r="K14" t="s">
         <v>60</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>855</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
         <v>358</v>
       </c>
@@ -42838,11 +42916,11 @@
       <c r="K15" t="s">
         <v>60</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
         <v>382</v>
       </c>
@@ -42876,11 +42954,11 @@
       <c r="K16" t="s">
         <v>60</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
         <v>403</v>
       </c>
@@ -42914,11 +42992,11 @@
       <c r="K17" t="s">
         <v>60</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="18" spans="1:12">
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
         <v>422</v>
       </c>
@@ -42952,11 +43030,11 @@
       <c r="K18" t="s">
         <v>59</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
         <v>443</v>
       </c>
@@ -42990,11 +43068,11 @@
       <c r="K19" t="s">
         <v>59</v>
       </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>855</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
         <v>467</v>
       </c>
@@ -43028,11 +43106,11 @@
       <c r="K20" t="s">
         <v>60</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="21" spans="1:12">
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
         <v>491</v>
       </c>
@@ -43066,11 +43144,11 @@
       <c r="K21" t="s">
         <v>59</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
         <v>514</v>
       </c>
@@ -43104,11 +43182,11 @@
       <c r="K22" t="s">
         <v>59</v>
       </c>
-      <c r="L22" t="s">
+      <c r="M22" t="s">
         <v>870</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
         <v>535</v>
       </c>
@@ -43142,11 +43220,11 @@
       <c r="K23" t="s">
         <v>59</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>873</v>
       </c>
     </row>
-    <row r="24" spans="1:12">
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
         <v>556</v>
       </c>
@@ -43180,11 +43258,11 @@
       <c r="K24" t="s">
         <v>60</v>
       </c>
-      <c r="L24" t="s">
+      <c r="M24" t="s">
         <v>877</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
         <v>576</v>
       </c>
@@ -43218,11 +43296,11 @@
       <c r="K25" t="s">
         <v>59</v>
       </c>
-      <c r="L25" t="s">
+      <c r="M25" t="s">
         <v>873</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
         <v>597</v>
       </c>
@@ -43256,11 +43334,11 @@
       <c r="K26" t="s">
         <v>60</v>
       </c>
-      <c r="L26" t="s">
+      <c r="M26" t="s">
         <v>879</v>
       </c>
     </row>
-    <row r="27" spans="1:12">
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
         <v>618</v>
       </c>
@@ -43294,11 +43372,11 @@
       <c r="K27" t="s">
         <v>59</v>
       </c>
-      <c r="L27" t="s">
+      <c r="M27" t="s">
         <v>884</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
         <v>637</v>
       </c>
@@ -43332,11 +43410,11 @@
       <c r="K28" t="s">
         <v>59</v>
       </c>
-      <c r="L28" t="s">
+      <c r="M28" t="s">
         <v>887</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
         <v>656</v>
       </c>
@@ -43370,11 +43448,11 @@
       <c r="K29" t="s">
         <v>59</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>889</v>
       </c>
     </row>
-    <row r="30" spans="1:12">
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
         <v>675</v>
       </c>
@@ -43408,11 +43486,11 @@
       <c r="K30" t="s">
         <v>59</v>
       </c>
-      <c r="L30" t="s">
+      <c r="M30" t="s">
         <v>896</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
         <v>693</v>
       </c>
@@ -43446,11 +43524,11 @@
       <c r="K31" t="s">
         <v>60</v>
       </c>
-      <c r="L31" t="s">
+      <c r="M31" t="s">
         <v>899</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:13">
       <c r="A32" t="s">
         <v>710</v>
       </c>
@@ -43484,11 +43562,11 @@
       <c r="K32" t="s">
         <v>60</v>
       </c>
-      <c r="L32" t="s">
+      <c r="M32" t="s">
         <v>884</v>
       </c>
     </row>
-    <row r="33" spans="1:12">
+    <row r="33" spans="1:13">
       <c r="A33" t="s">
         <v>729</v>
       </c>
@@ -43522,11 +43600,11 @@
       <c r="K33" t="s">
         <v>59</v>
       </c>
-      <c r="L33" t="s">
+      <c r="M33" t="s">
         <v>893</v>
       </c>
     </row>
-    <row r="34" spans="1:12">
+    <row r="34" spans="1:13">
       <c r="A34" t="s">
         <v>744</v>
       </c>
@@ -43560,11 +43638,11 @@
       <c r="K34" t="s">
         <v>60</v>
       </c>
-      <c r="L34" t="s">
+      <c r="M34" t="s">
         <v>889</v>
       </c>
     </row>
-    <row r="35" spans="1:12">
+    <row r="35" spans="1:13">
       <c r="A35" t="s">
         <v>762</v>
       </c>
@@ -43598,7 +43676,7 @@
       <c r="K35" t="s">
         <v>59</v>
       </c>
-      <c r="L35" t="s">
+      <c r="M35" t="s">
         <v>891</v>
       </c>
     </row>
@@ -48624,6 +48702,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -58668,6 +58747,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a945296-154d-4c56-a867-42b91b39e6cd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="33f4c322-9cc1-4712-bea0-1168c9f7fba8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010024A84FE412ECB7499435A3A398FE0BE1" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="eeb5e6dc7540569e23eb91fbf45376e8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a945296-154d-4c56-a867-42b91b39e6cd" xmlns:ns3="33f4c322-9cc1-4712-bea0-1168c9f7fba8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7af84f76c1ccc96e5ad5cdcf1bfcef5a" ns2:_="" ns3:_="">
     <xsd:import namespace="5a945296-154d-4c56-a867-42b91b39e6cd"/>
@@ -58862,27 +58961,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1325A7F-B636-4B33-8264-68F6F203A0B4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a945296-154d-4c56-a867-42b91b39e6cd"/>
+    <ds:schemaRef ds:uri="33f4c322-9cc1-4712-bea0-1168c9f7fba8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a945296-154d-4c56-a867-42b91b39e6cd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="33f4c322-9cc1-4712-bea0-1168c9f7fba8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DD21881-3B26-4282-A712-6E14D2513BAA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0AD3373-B6BE-4548-AE9E-8BC9167DB0F6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -58899,23 +58997,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DD21881-3B26-4282-A712-6E14D2513BAA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1325A7F-B636-4B33-8264-68F6F203A0B4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5a945296-154d-4c56-a867-42b91b39e6cd"/>
-    <ds:schemaRef ds:uri="33f4c322-9cc1-4712-bea0-1168c9f7fba8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix: days wo insurance in data and various other
</commit_message>
<xml_diff>
--- a/src/data/property_lob.xlsx
+++ b/src/data/property_lob.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3A99E19-88FE-4E92-B3F0-640B9A506CC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{349F2843-C293-4986-B75F-7D43B6F8FB41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Policy_Info" sheetId="1" r:id="rId1"/>
@@ -33714,7 +33714,9 @@
       <c r="U75" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V75" s="12"/>
+      <c r="V75" s="12">
+        <v>10</v>
+      </c>
       <c r="W75" s="12"/>
       <c r="X75" s="26"/>
       <c r="Y75" s="12">
@@ -33910,7 +33912,9 @@
       <c r="U77" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V77" s="12"/>
+      <c r="V77" s="12">
+        <v>10</v>
+      </c>
       <c r="W77" s="12"/>
       <c r="X77" s="26"/>
       <c r="Y77" s="12">
@@ -34008,7 +34012,9 @@
       <c r="U78" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V78" s="12"/>
+      <c r="V78" s="12">
+        <v>10</v>
+      </c>
       <c r="W78" s="12"/>
       <c r="X78" s="26"/>
       <c r="Y78" s="12">
@@ -34208,7 +34214,9 @@
       <c r="U80" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V80" s="12"/>
+      <c r="V80" s="12">
+        <v>10</v>
+      </c>
       <c r="W80" s="12"/>
       <c r="X80" s="26"/>
       <c r="Y80" s="12">
@@ -34306,7 +34314,9 @@
       <c r="U81" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V81" s="12"/>
+      <c r="V81" s="12">
+        <v>10</v>
+      </c>
       <c r="W81" s="12"/>
       <c r="X81" s="26"/>
       <c r="Y81" s="12">
@@ -34404,7 +34414,9 @@
       <c r="U82" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V82" s="12"/>
+      <c r="V82" s="12">
+        <v>10</v>
+      </c>
       <c r="W82" s="12"/>
       <c r="X82" s="26"/>
       <c r="Y82" s="12">
@@ -34502,7 +34514,9 @@
       <c r="U83" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V83" s="12"/>
+      <c r="V83" s="12">
+        <v>10</v>
+      </c>
       <c r="W83" s="12"/>
       <c r="X83" s="26"/>
       <c r="Y83" s="12">
@@ -34698,7 +34712,9 @@
       <c r="U85" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V85" s="12"/>
+      <c r="V85" s="12">
+        <v>10</v>
+      </c>
       <c r="W85" s="12"/>
       <c r="X85" s="26"/>
       <c r="Y85" s="12">
@@ -34896,7 +34912,9 @@
       <c r="U87" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V87" s="12"/>
+      <c r="V87" s="12">
+        <v>10</v>
+      </c>
       <c r="W87" s="12"/>
       <c r="X87" s="26"/>
       <c r="Y87" s="12">
@@ -34994,7 +35012,9 @@
       <c r="U88" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V88" s="12"/>
+      <c r="V88" s="12">
+        <v>10</v>
+      </c>
       <c r="W88" s="12"/>
       <c r="X88" s="26"/>
       <c r="Y88" s="12">
@@ -35192,7 +35212,9 @@
       <c r="U90" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V90" s="12"/>
+      <c r="V90" s="12">
+        <v>10</v>
+      </c>
       <c r="W90" s="12"/>
       <c r="X90" s="26"/>
       <c r="Y90" s="12">
@@ -35392,7 +35414,9 @@
       <c r="U92" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V92" s="12"/>
+      <c r="V92" s="12">
+        <v>10</v>
+      </c>
       <c r="W92" s="12"/>
       <c r="X92" s="26"/>
       <c r="Y92" s="12">
@@ -35490,7 +35514,9 @@
       <c r="U93" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V93" s="12"/>
+      <c r="V93" s="12">
+        <v>10</v>
+      </c>
       <c r="W93" s="12"/>
       <c r="X93" s="26"/>
       <c r="Y93" s="12">
@@ -35688,7 +35714,9 @@
       <c r="U95" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V95" s="12"/>
+      <c r="V95" s="12">
+        <v>10</v>
+      </c>
       <c r="W95" s="12"/>
       <c r="X95" s="26"/>
       <c r="Y95" s="12">
@@ -35886,7 +35914,9 @@
       <c r="U97" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V97" s="12"/>
+      <c r="V97" s="12">
+        <v>10</v>
+      </c>
       <c r="W97" s="12"/>
       <c r="X97" s="26"/>
       <c r="Y97" s="12">
@@ -36266,7 +36296,9 @@
       <c r="U101" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V101" s="12"/>
+      <c r="V101" s="12">
+        <v>10</v>
+      </c>
       <c r="W101" s="12"/>
       <c r="X101" s="26"/>
       <c r="Y101" s="12">
@@ -36364,7 +36396,9 @@
       <c r="U102" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V102" s="12"/>
+      <c r="V102" s="12">
+        <v>10</v>
+      </c>
       <c r="W102" s="12"/>
       <c r="X102" s="26"/>
       <c r="Y102" s="12">
@@ -36462,7 +36496,9 @@
       <c r="U103" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V103" s="12"/>
+      <c r="V103" s="12">
+        <v>10</v>
+      </c>
       <c r="W103" s="12"/>
       <c r="X103" s="26"/>
       <c r="Y103" s="12">
@@ -36660,7 +36696,9 @@
       <c r="U105" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V105" s="12"/>
+      <c r="V105" s="12">
+        <v>10</v>
+      </c>
       <c r="W105" s="12"/>
       <c r="X105" s="26"/>
       <c r="Y105" s="12">
@@ -36958,7 +36996,9 @@
       <c r="U108" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V108" s="12"/>
+      <c r="V108" s="12">
+        <v>10</v>
+      </c>
       <c r="W108" s="12"/>
       <c r="X108" s="26"/>
       <c r="Y108" s="12">
@@ -37156,7 +37196,9 @@
       <c r="U110" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V110" s="12"/>
+      <c r="V110" s="12">
+        <v>10</v>
+      </c>
       <c r="W110" s="12" t="s">
         <v>1213</v>
       </c>
@@ -37258,7 +37300,9 @@
       <c r="U111" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V111" s="12"/>
+      <c r="V111" s="12">
+        <v>10</v>
+      </c>
       <c r="W111" s="12"/>
       <c r="X111" s="26"/>
       <c r="Y111" s="12">
@@ -37356,7 +37400,9 @@
       <c r="U112" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V112" s="12"/>
+      <c r="V112" s="12">
+        <v>10</v>
+      </c>
       <c r="W112" s="12"/>
       <c r="X112" s="26"/>
       <c r="Y112" s="12">
@@ -37454,7 +37500,9 @@
       <c r="U113" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V113" s="12"/>
+      <c r="V113" s="12">
+        <v>10</v>
+      </c>
       <c r="W113" s="12"/>
       <c r="X113" s="26"/>
       <c r="Y113" s="12">
@@ -37750,7 +37798,9 @@
       <c r="U116" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V116" s="12"/>
+      <c r="V116" s="12">
+        <v>10</v>
+      </c>
       <c r="W116" s="12"/>
       <c r="X116" s="26"/>
       <c r="Y116" s="12">
@@ -37948,7 +37998,9 @@
       <c r="U118" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V118" s="12"/>
+      <c r="V118" s="12">
+        <v>10</v>
+      </c>
       <c r="W118" s="12"/>
       <c r="X118" s="26"/>
       <c r="Y118" s="12">
@@ -38046,7 +38098,9 @@
       <c r="U119" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V119" s="12"/>
+      <c r="V119" s="12">
+        <v>10</v>
+      </c>
       <c r="W119" s="12"/>
       <c r="X119" s="26"/>
       <c r="Y119" s="12">
@@ -38340,7 +38394,9 @@
       <c r="U122" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V122" s="12"/>
+      <c r="V122" s="12">
+        <v>10</v>
+      </c>
       <c r="W122" s="12"/>
       <c r="X122" s="26"/>
       <c r="Y122" s="12">
@@ -38540,7 +38596,9 @@
       <c r="U124" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V124" s="12"/>
+      <c r="V124" s="12">
+        <v>10</v>
+      </c>
       <c r="W124" s="12"/>
       <c r="X124" s="26"/>
       <c r="Y124" s="12">
@@ -38736,7 +38794,9 @@
       <c r="U126" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V126" s="12"/>
+      <c r="V126" s="12">
+        <v>10</v>
+      </c>
       <c r="W126" s="12"/>
       <c r="X126" s="26"/>
       <c r="Y126" s="12">
@@ -38932,7 +38992,9 @@
       <c r="U128" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V128" s="12"/>
+      <c r="V128" s="12">
+        <v>10</v>
+      </c>
       <c r="W128" s="12"/>
       <c r="X128" s="26"/>
       <c r="Y128" s="12">
@@ -39332,7 +39394,9 @@
       <c r="U132" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V132" s="12"/>
+      <c r="V132" s="12">
+        <v>10</v>
+      </c>
       <c r="W132" s="12"/>
       <c r="X132" s="26"/>
       <c r="Y132" s="12">
@@ -39430,7 +39494,9 @@
       <c r="U133" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V133" s="12"/>
+      <c r="V133" s="12">
+        <v>10</v>
+      </c>
       <c r="W133" s="12"/>
       <c r="X133" s="26"/>
       <c r="Y133" s="12">
@@ -39730,7 +39796,9 @@
       <c r="U136" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V136" s="12"/>
+      <c r="V136" s="12">
+        <v>10</v>
+      </c>
       <c r="W136" s="12"/>
       <c r="X136" s="26"/>
       <c r="Y136" s="12">
@@ -39928,7 +39996,9 @@
       <c r="U138" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V138" s="12"/>
+      <c r="V138" s="12">
+        <v>10</v>
+      </c>
       <c r="W138" s="12"/>
       <c r="X138" s="26"/>
       <c r="Y138" s="12">
@@ -40026,7 +40096,9 @@
       <c r="U139" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V139" s="12"/>
+      <c r="V139" s="12">
+        <v>10</v>
+      </c>
       <c r="W139" s="12"/>
       <c r="X139" s="26"/>
       <c r="Y139" s="12">
@@ -40324,7 +40396,9 @@
       <c r="U142" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V142" s="12"/>
+      <c r="V142" s="12">
+        <v>10</v>
+      </c>
       <c r="W142" s="12"/>
       <c r="X142" s="26"/>
       <c r="Y142" s="12">
@@ -40422,7 +40496,9 @@
       <c r="U143" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V143" s="12"/>
+      <c r="V143" s="12">
+        <v>10</v>
+      </c>
       <c r="W143" s="12"/>
       <c r="X143" s="26"/>
       <c r="Y143" s="12">
@@ -40520,7 +40596,9 @@
       <c r="U144" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V144" s="12"/>
+      <c r="V144" s="12">
+        <v>10</v>
+      </c>
       <c r="W144" s="12"/>
       <c r="X144" s="26"/>
       <c r="Y144" s="12">
@@ -40718,7 +40796,9 @@
       <c r="U146" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V146" s="12"/>
+      <c r="V146" s="12">
+        <v>10</v>
+      </c>
       <c r="W146" s="12"/>
       <c r="X146" s="26"/>
       <c r="Y146" s="12">
@@ -40916,7 +40996,9 @@
       <c r="U148" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V148" s="12"/>
+      <c r="V148" s="12">
+        <v>10</v>
+      </c>
       <c r="W148" s="12"/>
       <c r="X148" s="26"/>
       <c r="Y148" s="12">
@@ -41214,7 +41296,9 @@
       <c r="U151" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V151" s="12"/>
+      <c r="V151" s="12">
+        <v>10</v>
+      </c>
       <c r="W151" s="12"/>
       <c r="X151" s="26"/>
       <c r="Y151" s="12">
@@ -41312,7 +41396,9 @@
       <c r="U152" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V152" s="12"/>
+      <c r="V152" s="12">
+        <v>10</v>
+      </c>
       <c r="W152" s="12"/>
       <c r="X152" s="26"/>
       <c r="Y152" s="12">
@@ -41410,7 +41496,9 @@
       <c r="U153" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V153" s="12"/>
+      <c r="V153" s="12">
+        <v>10</v>
+      </c>
       <c r="W153" s="12"/>
       <c r="X153" s="26"/>
       <c r="Y153" s="12">
@@ -41508,7 +41596,9 @@
       <c r="U154" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V154" s="12"/>
+      <c r="V154" s="12">
+        <v>10</v>
+      </c>
       <c r="W154" s="12"/>
       <c r="X154" s="26"/>
       <c r="Y154" s="12">
@@ -41706,7 +41796,9 @@
       <c r="U156" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V156" s="12"/>
+      <c r="V156" s="12">
+        <v>10</v>
+      </c>
       <c r="W156" s="12"/>
       <c r="X156" s="26"/>
       <c r="Y156" s="12">
@@ -41804,7 +41896,9 @@
       <c r="U157" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V157" s="12"/>
+      <c r="V157" s="12">
+        <v>10</v>
+      </c>
       <c r="W157" s="12"/>
       <c r="X157" s="26"/>
       <c r="Y157" s="12">
@@ -42398,7 +42492,9 @@
       <c r="U163" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="V163" s="12"/>
+      <c r="V163" s="12">
+        <v>10</v>
+      </c>
       <c r="W163" s="12"/>
       <c r="X163" s="26"/>
       <c r="Y163" s="12">
@@ -43267,7 +43363,6 @@
       <c r="AI310" s="30"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM164" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
add: feature file loading logic more stricter
</commit_message>
<xml_diff>
--- a/src/data/property_lob.xlsx
+++ b/src/data/property_lob.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469A58D6-CB3B-4593-AD4D-60B15E41A6A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FA0C5EE-A450-48A7-8C9C-2D24A653E4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Policy_Info" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15108" uniqueCount="2099">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15112" uniqueCount="2099">
   <si>
     <t>Test ID</t>
   </si>
@@ -36159,15 +36159,33 @@
       </c>
       <c r="W99" s="12"/>
       <c r="X99" s="26"/>
-      <c r="Y99" s="12"/>
-      <c r="Z99" s="12"/>
-      <c r="AA99" s="12"/>
-      <c r="AB99" s="12"/>
-      <c r="AC99" s="12"/>
-      <c r="AD99" s="12"/>
-      <c r="AE99" s="12"/>
-      <c r="AF99" s="12"/>
-      <c r="AG99" s="12"/>
+      <c r="Y99" s="66">
+        <v>110</v>
+      </c>
+      <c r="Z99" s="66" t="s">
+        <v>1126</v>
+      </c>
+      <c r="AA99" s="66" t="s">
+        <v>1127</v>
+      </c>
+      <c r="AB99" s="66" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC99" s="66" t="s">
+        <v>59</v>
+      </c>
+      <c r="AD99" s="66">
+        <v>2016</v>
+      </c>
+      <c r="AE99" s="66">
+        <v>2017</v>
+      </c>
+      <c r="AF99" s="66">
+        <v>2017</v>
+      </c>
+      <c r="AG99" s="66">
+        <v>2020</v>
+      </c>
       <c r="AH99" s="12"/>
       <c r="AI99" s="12"/>
       <c r="AJ99" s="12"/>

</xml_diff>